<commit_message>
chore(data): daily refresh of list-source downloads
Updated: 2026-09-16T00:56:16+00:00
Total: 9, Success: 8, Failures: 1

Failures:
  - tjn-fsi: FetchError: TJN page rendered but no fsi_jurisdictions response captured. Endpoint or auth flow may have changed.
</commit_message>
<xml_diff>
--- a/public/downloads/fatf-jurisdictions.xlsx
+++ b/public/downloads/fatf-jurisdictions.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Data'!$A$1:$D$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Data'!$A$1:$D$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -511,7 +511,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-15T01:05:02+00:00</t>
+          <t>2026-09-16T00:54:15+00:00</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -600,12 +600,12 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Blacklist (Call for Action)</t>
+          <t>Greylist (Increased Monitoring)</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Democratic Republic of Korea</t>
+          <t>Angola</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
@@ -615,19 +615,19 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>https://www.fatf-gafi.org/en/publications/High-risk-and-other-monitored-jurisdictions/call-for-action-june-2026.html</t>
+          <t>https://www.fatf-gafi.org/en/publications/High-risk-and-other-monitored-jurisdictions/increased-monitoring-june-2026.html</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Blacklist (Call for Action)</t>
+          <t>Greylist (Increased Monitoring)</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Iran</t>
+          <t>Bolivia</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
@@ -637,19 +637,19 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>https://www.fatf-gafi.org/en/publications/High-risk-and-other-monitored-jurisdictions/call-for-action-june-2026.html</t>
+          <t>https://www.fatf-gafi.org/en/publications/High-risk-and-other-monitored-jurisdictions/increased-monitoring-june-2026.html</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Blacklist (Call for Action)</t>
+          <t>Greylist (Increased Monitoring)</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Myanmar</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>https://www.fatf-gafi.org/en/publications/High-risk-and-other-monitored-jurisdictions/call-for-action-june-2026.html</t>
+          <t>https://www.fatf-gafi.org/en/publications/High-risk-and-other-monitored-jurisdictions/increased-monitoring-june-2026.html</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Angola</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Cameroon</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Côte d'Ivoire</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Democratic Republic of the Congo</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Cameroon</t>
+          <t>Haiti</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Côte d'Ivoire</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Democratic Republic of the Congo</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Haiti</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Lao PDR</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Lebanon</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Kuwait</t>
+          <t>Monaco</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Lao PDR</t>
+          <t>Nepal</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Lebanon</t>
+          <t>Papua New Guinea</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Monaco</t>
+          <t>South Sudan</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Nepal</t>
+          <t>Syria</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Papua New Guinea</t>
+          <t>Venezuela</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>South Sudan</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Syria</t>
+          <t>Virgin Islands (UK)</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Venezuela</t>
+          <t>Yemen</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -1081,74 +1081,8 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Greylist (Increased Monitoring)</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Vietnam</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>19 June 2026</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>https://www.fatf-gafi.org/en/publications/High-risk-and-other-monitored-jurisdictions/increased-monitoring-june-2026.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>Greylist (Increased Monitoring)</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Virgin Islands (UK)</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>19 June 2026</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>https://www.fatf-gafi.org/en/publications/High-risk-and-other-monitored-jurisdictions/increased-monitoring-june-2026.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Greylist (Increased Monitoring)</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Yemen</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>19 June 2026</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>https://www.fatf-gafi.org/en/publications/High-risk-and-other-monitored-jurisdictions/increased-monitoring-june-2026.html</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D26"/>
+  <autoFilter ref="A1:D23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>